<commit_message>
up dzt in process
</commit_message>
<xml_diff>
--- a/SHET/DZT001/dtztnn.xlsx
+++ b/SHET/DZT001/dtztnn.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27932"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED0839A2-B0D6-4D5A-8A8D-3B3A4A417440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F6887D-9549-4E92-AF0D-AEBF2B3AC454}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,82 +23,82 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="26">
   <si>
-    <t>Уставка I&gt;, А</t>
+    <t>Iсраб, А</t>
+  </si>
+  <si>
+    <t>Δсраб, %</t>
+  </si>
+  <si>
+    <t>Iвозвр, А</t>
+  </si>
+  <si>
+    <t>Kвозвр</t>
+  </si>
+  <si>
+    <t>Iмин, А</t>
+  </si>
+  <si>
+    <t>Iмакс, А</t>
+  </si>
+  <si>
+    <t>Название таблицы</t>
+  </si>
+  <si>
+    <t>Тэг</t>
+  </si>
+  <si>
+    <t>Вход для проверки</t>
+  </si>
+  <si>
+    <t>Сигнал</t>
+  </si>
+  <si>
+    <t>Выход для контроля</t>
+  </si>
+  <si>
+    <t>—</t>
+  </si>
+  <si>
+    <t>ТС</t>
+  </si>
+  <si>
+    <t>ДТЗ/ ДТЗт: ИО фА</t>
+  </si>
+  <si>
+    <t>ДТЗ/ ДТЗт: ИО фВ</t>
+  </si>
+  <si>
+    <t>ДТЗ/ ДТЗт: ИО фС</t>
+  </si>
+  <si>
+    <t>Ia НН</t>
+  </si>
+  <si>
+    <t>Ib НН</t>
+  </si>
+  <si>
+    <t>Ic НН</t>
+  </si>
+  <si>
+    <t>X:33, X:34</t>
+  </si>
+  <si>
+    <t>X:35, X:36</t>
+  </si>
+  <si>
+    <t>X:37, X:38</t>
+  </si>
+  <si>
+    <t>dtztnn</t>
+  </si>
+  <si>
+    <t>Проверка тока срабатывания и коэффициента возврата ИО ДТЗт НН</t>
+  </si>
+  <si>
+    <t>Уставка Iср, о.е.</t>
   </si>
   <si>
     <t>Допустимый диапазон 3%</t>
-  </si>
-  <si>
-    <t>Iсраб, А</t>
-  </si>
-  <si>
-    <t>Δсраб, %</t>
-  </si>
-  <si>
-    <t>Iвозвр, А</t>
-  </si>
-  <si>
-    <t>Kвозвр</t>
-  </si>
-  <si>
-    <t>Iмин, А</t>
-  </si>
-  <si>
-    <t>Iмакс, А</t>
-  </si>
-  <si>
-    <t>Название таблицы</t>
-  </si>
-  <si>
-    <t>Тэг</t>
-  </si>
-  <si>
-    <t>Вход для проверки</t>
-  </si>
-  <si>
-    <t>Сигнал</t>
-  </si>
-  <si>
-    <t>Выход для контроля</t>
-  </si>
-  <si>
-    <t>—</t>
-  </si>
-  <si>
-    <t>ТС</t>
-  </si>
-  <si>
-    <t>ДТЗ/ ДТЗт: ИО фА</t>
-  </si>
-  <si>
-    <t>ДТЗ/ ДТЗт: ИО фВ</t>
-  </si>
-  <si>
-    <t>ДТЗ/ ДТЗт: ИО фС</t>
-  </si>
-  <si>
-    <t>Ia НН</t>
-  </si>
-  <si>
-    <t>Ib НН</t>
-  </si>
-  <si>
-    <t>Ic НН</t>
-  </si>
-  <si>
-    <t>X:33, X:34</t>
-  </si>
-  <si>
-    <t>X:35, X:36</t>
-  </si>
-  <si>
-    <t>X:37, X:38</t>
-  </si>
-  <si>
-    <t>dtztnn</t>
-  </si>
-  <si>
-    <t>Проверка тока срабатывания и коэффициента возврата ИО ДТЗт НН</t>
   </si>
 </sst>
 </file>
@@ -504,32 +504,32 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>12</v>
-      </c>
       <c r="D1" s="2" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="J1" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -538,10 +538,10 @@
       <c r="C2" s="3"/>
       <c r="D2" s="2"/>
       <c r="E2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -550,131 +550,131 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="s">
-        <v>15</v>
-      </c>
       <c r="C6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J7" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="I8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -706,18 +706,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>